<commit_message>
feat(buqi): persist ten-slot bazaar supply
</commit_message>
<xml_diff>
--- a/Design/Excel/GameHot/Datas/Buqi/BuqiMerchant.xlsx
+++ b/Design/Excel/GameHot/Datas/Buqi/BuqiMerchant.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BuqiMerchant" sheetId="1" r:id="Rdbd3ab9507274e74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BuqiMerchant" sheetId="1" r:id="R7b76ca0f95184da0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -265,6 +265,9 @@
       <x:c r="I1" t="str">
         <x:v>Slots</x:v>
       </x:c>
+      <x:c r="J1" t="str">
+        <x:v>Specialty</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
@@ -294,6 +297,9 @@
       <x:c r="I2" t="str">
         <x:v>(list#sep=|),BuqiMerchantSlotConfig</x:v>
       </x:c>
+      <x:c r="J2" t="str">
+        <x:v>BuqiMerchantSpecialty</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
@@ -322,6 +328,9 @@
       </x:c>
       <x:c r="I3" t="str">
         <x:v>offer slot constraints</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
+        <x:v>formal merchant supply specialty</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -350,6 +359,9 @@
       <x:c r="I4" t="str">
         <x:v>edge-a,Archetype,fast,S+M,Normal+Improved,attack,1,9,100,2|edge-b,Bridge,fast+chain,S,Normal+Improved,bridge,1,6,90,1|edge-c,Quality,fast,M+L,Improved+Fixed,core,4,9,70,1|edge-d,Counter,fast+burn,M,Normal+Improved,counter,4,9,60,1</x:v>
       </x:c>
+      <x:c r="J4" t="str">
+        <x:v>General</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5"/>
@@ -377,6 +389,9 @@
       <x:c r="I5" t="str">
         <x:v>bastion-a,Archetype,buffer,S+M,Normal+Improved,shield,1,9,100,2|bastion-b,Bridge,buffer,S,Normal+Improved,bridge,1,6,90,1|bastion-c,Stage,buffer,L,Improved+Fixed,finisher,7,9,70,1|bastion-d,Counter,buffer+heal,M,Normal+Improved,counter,4,9,60,1</x:v>
       </x:c>
+      <x:c r="J5" t="str">
+        <x:v>General</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6"/>
@@ -404,6 +419,9 @@
       <x:c r="I6" t="str">
         <x:v>spring-a,Archetype,heal,S+M,Normal+Improved,heal,1,9,100,2|spring-b,Bridge,heal,S,Normal+Improved,bridge,1,6,90,1|spring-c,Quality,heal,M+L,Improved+Fixed,regen,4,9,70,1|spring-d,Counter,heal+buffer,M,Normal+Improved,counter,4,9,60,1</x:v>
       </x:c>
+      <x:c r="J6" t="str">
+        <x:v>General</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7"/>
@@ -431,6 +449,9 @@
       <x:c r="I7" t="str">
         <x:v>measure-a,Size,fast+buffer+heal+chain,S,Normal+Improved,bridge,1,9,100,2|measure-b,Bridge,fast+buffer+heal,S,Normal+Improved,bridge,1,9,100,1|measure-c,Stage,shared,S,Normal+Improved,shared,1,6,70,1|measure-d,Quality,fast+buffer+heal,S,Improved,starter,1,6,60,1</x:v>
       </x:c>
+      <x:c r="J7" t="str">
+        <x:v>NonWeaponOnly</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8"/>
@@ -458,6 +479,9 @@
       <x:c r="I8" t="str">
         <x:v>gap-a,Counter,fast+buffer+heal,M,Normal+Improved,counter,4,9,110,2|gap-b,Counter,poison+freeze+overload,S+M,Normal+Improved,counter,1,9,90,1|gap-c,Quality,shared,M,Improved+Fixed,counter,4,9,70,1|gap-d,Stage,fast+buffer+heal,M,Improved,pivot,4,9,60,1</x:v>
       </x:c>
+      <x:c r="J8" t="str">
+        <x:v>General</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9"/>
@@ -485,6 +509,9 @@
       <x:c r="I9" t="str">
         <x:v>ledger-a,Economy,fast+buffer+heal+shared,S,Normal+Improved,economy,7,9,120,2|ledger-b,Size,fast+buffer+heal,S,Normal,starter,1,9,80,1|ledger-c,Quality,shared,S,Improved+Fixed,economy,7,9,70,1|ledger-d,Counter,overload,S,Normal+Improved,counter,1,9,50,1</x:v>
       </x:c>
+      <x:c r="J9" t="str">
+        <x:v>General</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10"/>
@@ -512,6 +539,9 @@
       <x:c r="I10" t="str">
         <x:v>grades-a,Quality,fast+buffer+heal,M,Improved,core,4,9,100,2|grades-b,Quality,chain+poison+burn+freeze+overload,M,Improved,core,4,9,80,1|grades-c,Stage,fast+buffer+heal,M,Fixed,pivot,7,9,60,1|grades-d,Size,shared,M,Improved+Fixed,counter,4,9,50,1</x:v>
       </x:c>
+      <x:c r="J10" t="str">
+        <x:v>General</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11"/>
@@ -539,6 +569,9 @@
       <x:c r="I11" t="str">
         <x:v>summit-a,Stage,fast+buffer+heal,L,Improved+Fixed,finisher,7,9,120,2|summit-b,Size,poison+burn+freeze,L,Improved+Fixed,finisher,7,9,90,1|summit-c,Economy,fast+buffer+heal+shared,S,Improved+Fixed,economy,7,9,70,1|summit-d,Quality,fast+buffer+heal,L,Fixed,finisher,7,9,50,1</x:v>
       </x:c>
+      <x:c r="J11" t="str">
+        <x:v>General</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>